<commit_message>
autobump ms.js ?v=454 for PHOTO-ORDER-1 + Aug-2026 blur-lane swap costing sheet
</commit_message>
<xml_diff>
--- a/AI_PHOTO_COST_MODEL.xlsx
+++ b/AI_PHOTO_COST_MODEL.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per-photo model" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Switch Test Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing (Aug 2026) swap" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -27,7 +28,7 @@
     <numFmt numFmtId="167" formatCode="$0.0000"/>
     <numFmt numFmtId="168" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -91,8 +92,16 @@
       <name val="Arial"/>
       <color rgb="000000FF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -114,6 +123,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
   </fills>
@@ -165,7 +179,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -273,6 +287,8 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -945,14 +961,7 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="17"/>
-    <row r="13" ht="15" customHeight="1" s="17">
-      <c r="A13" s="25" t="inlineStr">
-        <is>
-          <t>GLM sovereignty note: photos of users' homes/cars routed to a China-hosted provider is a POPIA + trust-brand decision, not just a price one (see AI_SOVEREIGNTY_PHYSICAL_LAYER_DECISION_2026-07-09.md). OpenRouter hosting mitigates jurisdiction but adds a middleman.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14"/>
+    <row r="13" ht="15" customHeight="1" s="17"/>
     <row r="15" ht="15" customHeight="1" s="17"/>
     <row r="16">
       <c r="A16" s="26" t="inlineStr">
@@ -1774,4 +1783,383 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" style="17" min="1" max="1"/>
+    <col width="8" customWidth="1" style="17" min="2" max="2"/>
+    <col width="8" customWidth="1" style="17" min="3" max="3"/>
+    <col width="12" customWidth="1" style="17" min="4" max="4"/>
+    <col width="12" customWidth="1" style="17" min="5" max="5"/>
+    <col width="12" customWidth="1" style="17" min="6" max="6"/>
+    <col width="10" customWidth="1" style="17" min="7" max="7"/>
+    <col width="14" customWidth="1" style="17" min="8" max="8"/>
+    <col width="60" customWidth="1" style="17" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>Blur-lane swap costing — 19 Aug 2026 · same per-photo assumptions as 'Per-photo model' sheet · RUL-031</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B2" s="40" t="inlineStr">
+        <is>
+          <t>$/M in</t>
+        </is>
+      </c>
+      <c r="C2" s="40" t="inlineStr">
+        <is>
+          <t>$/M out</t>
+        </is>
+      </c>
+      <c r="D2" s="40" t="inlineStr">
+        <is>
+          <t>$ clean photo</t>
+        </is>
+      </c>
+      <c r="E2" s="40" t="inlineStr">
+        <is>
+          <t>$ redacted</t>
+        </is>
+      </c>
+      <c r="F2" s="40" t="inlineStr">
+        <is>
+          <t>$ avg photo</t>
+        </is>
+      </c>
+      <c r="G2" s="40" t="inlineStr">
+        <is>
+          <t>$ / 1,000</t>
+        </is>
+      </c>
+      <c r="H2" s="40" t="inlineStr">
+        <is>
+          <t>$ Year-1 (197k)</t>
+        </is>
+      </c>
+      <c r="I2" s="40" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>OpenAI gpt-5.6-terra (TODAY)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.00587</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.01446</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.00878</v>
+      </c>
+      <c r="G3" t="n">
+        <v>8.779999999999999</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1729</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>current standing lane — the one that just failed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Anthropic Sonnet 4.6 (failover)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>15</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.008569999999999999</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.02104</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.01278</v>
+      </c>
+      <c r="G4" t="n">
+        <v>12.78</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2518</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>pre-14-Aug lane — failed the same way</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Scaleway mistral-medium-3.5 (net)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="C5" t="n">
+        <v>9.369999999999999</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.00458</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.01128</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.00685</v>
+      </c>
+      <c r="G5" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1349</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>derived from 0.781x baseline multiple</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Gemini 3.7 Flash</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.00077</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.00186</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.00114</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="H6" t="n">
+        <v>224</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>OUT price ESTIMATE — verify at ai.google.dev before any switch</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Grok 4.1 Fast</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.00053</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.00129</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.00079</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="H7" t="n">
+        <v>155</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>xAI volume tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Grok 4.6</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.00539</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.01314</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.00801</v>
+      </c>
+      <c r="G8" t="n">
+        <v>8.01</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1579</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>xAI flagship</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Qwen3-VL (EU host)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.00108</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.00263</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H9" t="n">
+        <v>316</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ESTIMATE — no EU-host price sheet yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Local CV detector (YOLO+OCR)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>$0 marginal; our CPU</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CANARY: Gemini scans+refines, terra verifies every redaction (their own Switch Test Plan step 2 — a weak scanner degrades to more verify rounds, never to a leak)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>0.00077</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.00696</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.00278</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="H11" t="n">
+        <v>548</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>zero-leak-risk first step</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Context: gate history — Haiku FAILED this task pre-7-Jul (missed plates); 'cheapest' already lost once. Recall on the 30-photo eval set must be 100% BEFORE any traffic (Switch Test Plan). Gemini uniquely returns segmentation MASKS (surgical, not rectangles); Qwen3-VL is grounding-trained; Grok/Mistral are general LLMs like the two that failed. Local CV = $0/call, needs ~2 days + eval.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Nightly checkpoint Wed 08/26/2026  5:30:03.30 (auto, no deploy)
</commit_message>
<xml_diff>
--- a/AI_PHOTO_COST_MODEL.xlsx
+++ b/AI_PHOTO_COST_MODEL.xlsx
@@ -1791,7 +1791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" style="17" min="1" max="1"/>
@@ -1860,302 +1860,423 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>OpenAI gpt-5.6-terra (TODAY)</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="16" t="n">
         <v>0.00587</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="16" t="n">
         <v>0.01446</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="16" t="n">
         <v>0.00878</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="16" t="n">
         <v>8.779999999999999</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="16" t="n">
         <v>1729</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="16" t="inlineStr">
         <is>
           <t>current standing lane — the one that just failed</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Anthropic Sonnet 4.6 (failover)</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="16" t="n">
         <v>0.008569999999999999</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="16" t="n">
         <v>0.02104</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="16" t="n">
         <v>0.01278</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="16" t="n">
         <v>12.78</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="16" t="n">
         <v>2518</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="16" t="inlineStr">
         <is>
           <t>pre-14-Aug lane — failed the same way</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Scaleway mistral-medium-3.5 (net)</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="16" t="n">
         <v>1.56</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="16" t="n">
         <v>9.369999999999999</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="16" t="n">
         <v>0.00458</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="16" t="n">
         <v>0.01128</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="16" t="n">
         <v>0.00685</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="16" t="n">
         <v>6.85</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="16" t="n">
         <v>1349</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="16" t="inlineStr">
         <is>
           <t>derived from 0.781x baseline multiple</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>Gemini 3.7 Flash</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="C6" t="n">
+      <c r="B6" s="16" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="E6" s="16" t="n">
+        <v>0.00418</v>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>0.00269</v>
+      </c>
+      <c r="G6" s="16" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="H6" s="16" t="n">
+        <v>529</v>
+      </c>
+      <c r="I6" s="16" t="inlineStr">
+        <is>
+          <t>CORRECTED 26 Aug 2026 — first-party ai.google.dev STANDARD tier $0.75/$3.75 (the 19 Aug row used $0.375 = the BATCH rate, and a $1.50 out ESTIMATE). Was modelled $224/yr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Grok 4.1 Fast</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>0.00053</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>0.00129</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>0.00079</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>155</v>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>xAI volume tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Grok 4.6</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>0.00539</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>0.01314</v>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>0.00801</v>
+      </c>
+      <c r="G8" s="16" t="n">
+        <v>8.01</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <v>1579</v>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>xAI flagship</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Qwen3-VL (EU host)</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>0.00108</v>
+      </c>
+      <c r="E9" s="16" t="n">
+        <v>0.00263</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="G9" s="16" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H9" s="16" t="n">
+        <v>316</v>
+      </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>ESTIMATE — no EU-host price sheet yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Local CV detector (YOLO+OCR)</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>$0 marginal; our CPU</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>CANARY: Gemini scans+refines, terra verifies every redaction (their own Switch Test Plan step 2 — a weak scanner degrades to more verify rounds, never to a leak)</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr"/>
+      <c r="C11" s="16" t="inlineStr"/>
+      <c r="D11" s="16" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="E11" s="16" t="n">
+        <v>0.008449999999999999</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>0.00429</v>
+      </c>
+      <c r="G11" s="16" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="H11" s="16" t="n">
+        <v>845</v>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>CORRECTED 26 Aug 2026 on first-party prices. Was modelled $548/yr. Still the cheapest zero-leak-risk step: vs terra-only $1,729/yr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Context: gate history — Haiku FAILED this task pre-7-Jul (missed plates); 'cheapest' already lost once. Recall on the 30-photo eval set must be 100% BEFORE any traffic (Switch Test Plan). Gemini uniquely returns segmentation MASKS (surgical, not rectangles); Qwen3-VL is grounding-trained; Grok/Mistral are general LLMs like the two that failed. Local CV = $0/call, needs ~2 days + eval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PRICE STEP — Gemini introductory pricing EXPIRES 31 Dec 2026; from 1 Jan 2027 standard is $1.50 in / $7.50 out (2x). Same assumptions, re-costed:</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>$/M in</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>$/M out</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>$ clean photo</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>$ redacted</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>$ avg photo</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>$ / 1,000</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>$ Year-1 (197k)</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Gemini 3.7 Flash (from 1 Jan 2027)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
         <v>1.5</v>
       </c>
-      <c r="D6" t="n">
-        <v>0.00077</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.00186</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.00114</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="H6" t="n">
-        <v>224</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>OUT price ESTIMATE — verify at ai.google.dev before any switch</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Grok 4.1 Fast</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.00053</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.00129</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.00079</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.79</v>
-      </c>
-      <c r="H7" t="n">
-        <v>155</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>xAI volume tier</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Grok 4.6</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" t="n">
-        <v>6</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.00539</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0.01314</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0.00801</v>
-      </c>
-      <c r="G8" t="n">
-        <v>8.01</v>
-      </c>
-      <c r="H8" t="n">
-        <v>1579</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>xAI flagship</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Qwen3-VL (EU host)</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="C9" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.00108</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.00263</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.0016</v>
-      </c>
-      <c r="G9" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="H9" t="n">
-        <v>316</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>ESTIMATE — no EU-host price sheet yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Local CV detector (YOLO+OCR)</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>$0 marginal; our CPU</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>CANARY: Gemini scans+refines, terra verifies every redaction (their own Switch Test Plan step 2 — a weak scanner degrades to more verify rounds, never to a leak)</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="n">
-        <v>0.00077</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0.00696</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0.00278</v>
-      </c>
-      <c r="G11" t="n">
-        <v>2.78</v>
-      </c>
-      <c r="H11" t="n">
-        <v>548</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>zero-leak-risk first step</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Context: gate history — Haiku FAILED this task pre-7-Jul (missed plates); 'cheapest' already lost once. Recall on the 30-photo eval set must be 100% BEFORE any traffic (Switch Test Plan). Gemini uniquely returns segmentation MASKS (surgical, not rectangles); Qwen3-VL is grounding-trained; Grok/Mistral are general LLMs like the two that failed. Local CV = $0/call, needs ~2 days + eval.</t>
+      <c r="C17" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.00835</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.00537</v>
+      </c>
+      <c r="G17" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1058</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>full switch at post-intro pricing</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CANARY (gemini scan+refine, terra verify) — from 1 Jan 2027</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C18" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.0032</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.01102</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.00637</v>
+      </c>
+      <c r="G18" t="n">
+        <v>6.37</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1256</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>canary at post-intro pricing; margin vs terra-only ($1,729) narrows sharply — decide before the step whether to promote to full switch or move to the local CV detector ($0 marginal).</t>
         </is>
       </c>
     </row>

</xml_diff>